<commit_message>
v7: four headline models on a single jurisdiction basis, zero-vs-missing audit
Fix CANON_JUR = K_REACH as the one cross-jurisdiction basis (only projection
matching both K-REACH and US OSHA with zero loss; not chosen for performance).
Other jurisdictions, missing-data protocols and CT arms stay as supplementary
rows with 대표 = 0, so switching the basis needs no re-run. Each output dir now
carries 규제처리_명시.md with the statutory basis and full projection tables.

Add audit_zero_vs_missing.py: exactly two columns had missing frozen into 0 at
build time (f_pct_surf_total, f_surf_anionic_nonionic; 281 rows each, unknown
composition) via the `x or 0.0` idiom in the version-pinned build_input_v5.
New native_복원 protocol restores them model-side; nan0 kept only as the v6
reproduction control, which still locks to 1e-9.

Untrack the Word reports (*.docx) — internal review material, not for sharing.
Rewrite README in English.
</commit_message>
<xml_diff>
--- a/04_모델산출물/v7_성분모델/지표_성분모델.xlsx
+++ b/04_모델산출물/v7_성분모델/지표_성분모델.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="물질_라벨대장" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'성분모델'!$A$1:$AL$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'성분모델'!$A$1:$AM$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'물질_라벨대장'!$A$1:$J$662</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,1739 +417,1780 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL13"/>
+  <dimension ref="A1:AM13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>대표</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>단위</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>endpoint</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>관할</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>피처</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>결측처리</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>CT</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>n</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>양성</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>유병률</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>roc_auc</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>roc_auc_sd</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>pr_auc</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>pr_auc_sd</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>f1_pos</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>f1_pos_sd</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>f1_neg</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>f1_macro</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>precision</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>recall</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>specificity</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>MCC</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>BA</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>accuracy</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>tp</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>fp</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>fn</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>tn</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>F1_최적임계값_참고_seed4</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>최적임계값_참고_seed4</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>f1_neg_sd</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>f1_macro_sd</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>precision_sd</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>recall_sd</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>specificity_sd</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>MCC_sd</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>BA_sd</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>accuracy_sd</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>골격그룹수</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>성분</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>eye</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>UN_GHS+K_REACH+US_OSHA</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>구조</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>nan0</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>398</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>177</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>0.4447</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>0.7557</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>0.0067</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>0.7086</v>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>0.0121</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>0.6794</v>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
         <v>0.0109</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>0.7547</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>0.7171</v>
       </c>
-      <c r="R2" t="n">
+      <c r="S2" t="n">
         <v>0.698</v>
       </c>
-      <c r="S2" t="n">
+      <c r="T2" t="n">
         <v>0.6621</v>
       </c>
-      <c r="T2" t="n">
+      <c r="U2" t="n">
         <v>0.7701</v>
       </c>
-      <c r="U2" t="n">
+      <c r="V2" t="n">
         <v>0.4351</v>
       </c>
-      <c r="V2" t="n">
+      <c r="W2" t="n">
         <v>0.7161</v>
       </c>
-      <c r="W2" t="n">
+      <c r="X2" t="n">
         <v>0.7221</v>
       </c>
-      <c r="X2" t="n">
+      <c r="Y2" t="n">
         <v>117.2</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="Z2" t="n">
         <v>50.8</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="AA2" t="n">
         <v>59.8</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AB2" t="n">
         <v>170.2</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AC2" t="n">
         <v>0.7244</v>
       </c>
-      <c r="AC2" t="n">
+      <c r="AD2" t="n">
         <v>0.436</v>
       </c>
-      <c r="AD2" t="n">
+      <c r="AE2" t="n">
         <v>0.0121</v>
       </c>
-      <c r="AE2" t="n">
+      <c r="AF2" t="n">
         <v>0.011</v>
       </c>
-      <c r="AF2" t="n">
+      <c r="AG2" t="n">
         <v>0.0175</v>
       </c>
-      <c r="AG2" t="n">
+      <c r="AH2" t="n">
         <v>0.0135</v>
       </c>
-      <c r="AH2" t="n">
+      <c r="AI2" t="n">
         <v>0.0201</v>
       </c>
-      <c r="AI2" t="n">
+      <c r="AJ2" t="n">
         <v>0.0223</v>
       </c>
-      <c r="AJ2" t="n">
+      <c r="AK2" t="n">
         <v>0.0107</v>
       </c>
-      <c r="AK2" t="n">
+      <c r="AL2" t="n">
         <v>0.0113</v>
       </c>
-      <c r="AL2" t="n">
+      <c r="AM2" t="n">
         <v>168</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="n">
+        <v>0</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>성분</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>eye</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>UN_GHS+K_REACH+US_OSHA</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>구조+지문</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>nan0</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>398</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>177</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>0.4447</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>0.7554</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>0.0065</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>0.7065</v>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>0.0025</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>0.6816</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>0.0175</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>0.7502</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>0.7159</v>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>0.6893</v>
       </c>
-      <c r="S3" t="n">
+      <c r="T3" t="n">
         <v>0.6746</v>
       </c>
-      <c r="T3" t="n">
+      <c r="U3" t="n">
         <v>0.7566000000000001</v>
       </c>
-      <c r="U3" t="n">
+      <c r="V3" t="n">
         <v>0.4323</v>
       </c>
-      <c r="V3" t="n">
+      <c r="W3" t="n">
         <v>0.7156</v>
       </c>
-      <c r="W3" t="n">
+      <c r="X3" t="n">
         <v>0.7201</v>
       </c>
-      <c r="X3" t="n">
+      <c r="Y3" t="n">
         <v>119.4</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="Z3" t="n">
         <v>53.8</v>
       </c>
-      <c r="Z3" t="n">
+      <c r="AA3" t="n">
         <v>57.6</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="AB3" t="n">
         <v>167.2</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AC3" t="n">
         <v>0.7243000000000001</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="AD3" t="n">
         <v>0.48</v>
       </c>
-      <c r="AD3" t="n">
+      <c r="AE3" t="n">
         <v>0.0061</v>
       </c>
-      <c r="AE3" t="n">
+      <c r="AF3" t="n">
         <v>0.0117</v>
       </c>
-      <c r="AF3" t="n">
+      <c r="AG3" t="n">
         <v>0.0054</v>
       </c>
-      <c r="AG3" t="n">
+      <c r="AH3" t="n">
         <v>0.0306</v>
       </c>
-      <c r="AH3" t="n">
+      <c r="AI3" t="n">
         <v>0.0067</v>
       </c>
-      <c r="AI3" t="n">
+      <c r="AJ3" t="n">
         <v>0.0235</v>
       </c>
-      <c r="AJ3" t="n">
+      <c r="AK3" t="n">
         <v>0.0126</v>
       </c>
-      <c r="AK3" t="n">
+      <c r="AL3" t="n">
         <v>0.0106</v>
       </c>
-      <c r="AL3" t="n">
+      <c r="AM3" t="n">
         <v>168</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="n">
+        <v>0</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>성분</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>eye</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>UN_GHS+K_REACH+US_OSHA</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>구조</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>398</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>177</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>0.4447</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>0.7537</v>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>0.006</v>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>0.7045</v>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>0.0107</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>0.674</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>0.0049</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>0.7508</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>0.7124</v>
       </c>
-      <c r="R4" t="n">
+      <c r="S4" t="n">
         <v>0.6929</v>
       </c>
-      <c r="S4" t="n">
+      <c r="T4" t="n">
         <v>0.6565</v>
       </c>
-      <c r="T4" t="n">
+      <c r="U4" t="n">
         <v>0.7665</v>
       </c>
-      <c r="U4" t="n">
+      <c r="V4" t="n">
         <v>0.4259</v>
       </c>
-      <c r="V4" t="n">
+      <c r="W4" t="n">
         <v>0.7115</v>
       </c>
-      <c r="W4" t="n">
+      <c r="X4" t="n">
         <v>0.7176</v>
       </c>
-      <c r="X4" t="n">
+      <c r="Y4" t="n">
         <v>116.2</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="Z4" t="n">
         <v>51.6</v>
       </c>
-      <c r="Z4" t="n">
+      <c r="AA4" t="n">
         <v>60.8</v>
       </c>
-      <c r="AA4" t="n">
+      <c r="AB4" t="n">
         <v>169.4</v>
       </c>
-      <c r="AB4" t="n">
+      <c r="AC4" t="n">
         <v>0.7154</v>
       </c>
-      <c r="AC4" t="n">
+      <c r="AD4" t="n">
         <v>0.425</v>
       </c>
-      <c r="AD4" t="n">
+      <c r="AE4" t="n">
         <v>0.0097</v>
       </c>
-      <c r="AE4" t="n">
+      <c r="AF4" t="n">
         <v>0.0069</v>
       </c>
-      <c r="AF4" t="n">
+      <c r="AG4" t="n">
         <v>0.0149</v>
       </c>
-      <c r="AG4" t="n">
+      <c r="AH4" t="n">
         <v>0.009299999999999999</v>
       </c>
-      <c r="AH4" t="n">
+      <c r="AI4" t="n">
         <v>0.0191</v>
       </c>
-      <c r="AI4" t="n">
+      <c r="AJ4" t="n">
         <v>0.0145</v>
       </c>
-      <c r="AJ4" t="n">
+      <c r="AK4" t="n">
         <v>0.0064</v>
       </c>
-      <c r="AK4" t="n">
+      <c r="AL4" t="n">
         <v>0.0077</v>
       </c>
-      <c r="AL4" t="n">
+      <c r="AM4" t="n">
         <v>168</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>성분</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>eye</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>UN_GHS+K_REACH+US_OSHA</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>구조+지문</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>398</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>177</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>0.4447</v>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>0.7543</v>
       </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>0.0072</v>
       </c>
-      <c r="L5" t="n">
+      <c r="M5" t="n">
         <v>0.7033</v>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>0.0048</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>0.6826</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>0.021</v>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>0.7544</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
         <v>0.7185</v>
       </c>
-      <c r="R5" t="n">
+      <c r="S5" t="n">
         <v>0.6958</v>
       </c>
-      <c r="S5" t="n">
+      <c r="T5" t="n">
         <v>0.6701</v>
       </c>
-      <c r="T5" t="n">
+      <c r="U5" t="n">
         <v>0.7655999999999999</v>
       </c>
-      <c r="U5" t="n">
+      <c r="V5" t="n">
         <v>0.4376</v>
       </c>
-      <c r="V5" t="n">
+      <c r="W5" t="n">
         <v>0.7178</v>
       </c>
-      <c r="W5" t="n">
+      <c r="X5" t="n">
         <v>0.7231</v>
       </c>
-      <c r="X5" t="n">
+      <c r="Y5" t="n">
         <v>118.6</v>
       </c>
-      <c r="Y5" t="n">
+      <c r="Z5" t="n">
         <v>51.8</v>
       </c>
-      <c r="Z5" t="n">
+      <c r="AA5" t="n">
         <v>58.4</v>
       </c>
-      <c r="AA5" t="n">
+      <c r="AB5" t="n">
         <v>169.2</v>
       </c>
-      <c r="AB5" t="n">
+      <c r="AC5" t="n">
         <v>0.7278</v>
       </c>
-      <c r="AC5" t="n">
+      <c r="AD5" t="n">
         <v>0.476</v>
       </c>
-      <c r="AD5" t="n">
+      <c r="AE5" t="n">
         <v>0.0107</v>
       </c>
-      <c r="AE5" t="n">
+      <c r="AF5" t="n">
         <v>0.0157</v>
       </c>
-      <c r="AF5" t="n">
+      <c r="AG5" t="n">
         <v>0.0123</v>
       </c>
-      <c r="AG5" t="n">
+      <c r="AH5" t="n">
         <v>0.0298</v>
       </c>
-      <c r="AH5" t="n">
+      <c r="AI5" t="n">
         <v>0.0059</v>
       </c>
-      <c r="AI5" t="n">
+      <c r="AJ5" t="n">
         <v>0.031</v>
       </c>
-      <c r="AJ5" t="n">
+      <c r="AK5" t="n">
         <v>0.0161</v>
       </c>
-      <c r="AK5" t="n">
+      <c r="AL5" t="n">
         <v>0.0147</v>
       </c>
-      <c r="AL5" t="n">
+      <c r="AM5" t="n">
         <v>168</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>성분</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>eye</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>EU_CLP</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>구조</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>nan0</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>338</v>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>116</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>0.3432</v>
       </c>
-      <c r="J6" t="n">
+      <c r="K6" t="n">
         <v>0.801</v>
       </c>
-      <c r="K6" t="n">
+      <c r="L6" t="n">
         <v>0.004</v>
       </c>
-      <c r="L6" t="n">
+      <c r="M6" t="n">
         <v>0.676</v>
       </c>
-      <c r="M6" t="n">
+      <c r="N6" t="n">
         <v>0.0121</v>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>0.6392</v>
       </c>
-      <c r="O6" t="n">
+      <c r="P6" t="n">
         <v>0.0159</v>
       </c>
-      <c r="P6" t="n">
+      <c r="Q6" t="n">
         <v>0.8205</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="R6" t="n">
         <v>0.7299</v>
       </c>
-      <c r="R6" t="n">
+      <c r="S6" t="n">
         <v>0.6614</v>
       </c>
-      <c r="S6" t="n">
+      <c r="T6" t="n">
         <v>0.619</v>
       </c>
-      <c r="T6" t="n">
+      <c r="U6" t="n">
         <v>0.8342000000000001</v>
       </c>
-      <c r="U6" t="n">
+      <c r="V6" t="n">
         <v>0.4609</v>
       </c>
-      <c r="V6" t="n">
+      <c r="W6" t="n">
         <v>0.7266</v>
       </c>
-      <c r="W6" t="n">
+      <c r="X6" t="n">
         <v>0.7604</v>
       </c>
-      <c r="X6" t="n">
+      <c r="Y6" t="n">
         <v>71.8</v>
       </c>
-      <c r="Y6" t="n">
+      <c r="Z6" t="n">
         <v>36.8</v>
       </c>
-      <c r="Z6" t="n">
+      <c r="AA6" t="n">
         <v>44.2</v>
       </c>
-      <c r="AA6" t="n">
+      <c r="AB6" t="n">
         <v>185.2</v>
       </c>
-      <c r="AB6" t="n">
+      <c r="AC6" t="n">
         <v>0.6912</v>
       </c>
-      <c r="AC6" t="n">
+      <c r="AD6" t="n">
         <v>0.356</v>
       </c>
-      <c r="AD6" t="n">
+      <c r="AE6" t="n">
         <v>0.0069</v>
       </c>
-      <c r="AE6" t="n">
+      <c r="AF6" t="n">
         <v>0.0106</v>
       </c>
-      <c r="AF6" t="n">
+      <c r="AG6" t="n">
         <v>0.0156</v>
       </c>
-      <c r="AG6" t="n">
+      <c r="AH6" t="n">
         <v>0.0254</v>
       </c>
-      <c r="AH6" t="n">
+      <c r="AI6" t="n">
         <v>0.0133</v>
       </c>
-      <c r="AI6" t="n">
+      <c r="AJ6" t="n">
         <v>0.0206</v>
       </c>
-      <c r="AJ6" t="n">
+      <c r="AK6" t="n">
         <v>0.0111</v>
       </c>
-      <c r="AK6" t="n">
+      <c r="AL6" t="n">
         <v>0.0089</v>
       </c>
-      <c r="AL6" t="n">
+      <c r="AM6" t="n">
         <v>153</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>성분</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>eye</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>EU_CLP</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>구조+지문</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>nan0</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>338</v>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>116</v>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>0.3432</v>
       </c>
-      <c r="J7" t="n">
+      <c r="K7" t="n">
         <v>0.8024</v>
       </c>
-      <c r="K7" t="n">
+      <c r="L7" t="n">
         <v>0.004</v>
       </c>
-      <c r="L7" t="n">
+      <c r="M7" t="n">
         <v>0.6713</v>
       </c>
-      <c r="M7" t="n">
+      <c r="N7" t="n">
         <v>0.0083</v>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>0.6137</v>
       </c>
-      <c r="O7" t="n">
+      <c r="P7" t="n">
         <v>0.0129</v>
       </c>
-      <c r="P7" t="n">
+      <c r="Q7" t="n">
         <v>0.8206</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="R7" t="n">
         <v>0.7171999999999999</v>
       </c>
-      <c r="R7" t="n">
+      <c r="S7" t="n">
         <v>0.6688</v>
       </c>
-      <c r="S7" t="n">
+      <c r="T7" t="n">
         <v>0.5672</v>
       </c>
-      <c r="T7" t="n">
+      <c r="U7" t="n">
         <v>0.8532</v>
       </c>
-      <c r="U7" t="n">
+      <c r="V7" t="n">
         <v>0.4394</v>
       </c>
-      <c r="V7" t="n">
+      <c r="W7" t="n">
         <v>0.7102000000000001</v>
       </c>
-      <c r="W7" t="n">
+      <c r="X7" t="n">
         <v>0.755</v>
       </c>
-      <c r="X7" t="n">
+      <c r="Y7" t="n">
         <v>65.8</v>
       </c>
-      <c r="Y7" t="n">
+      <c r="Z7" t="n">
         <v>32.6</v>
       </c>
-      <c r="Z7" t="n">
+      <c r="AA7" t="n">
         <v>50.2</v>
       </c>
-      <c r="AA7" t="n">
+      <c r="AB7" t="n">
         <v>189.4</v>
       </c>
-      <c r="AB7" t="n">
+      <c r="AC7" t="n">
         <v>0.6939</v>
       </c>
-      <c r="AC7" t="n">
+      <c r="AD7" t="n">
         <v>0.297</v>
       </c>
-      <c r="AD7" t="n">
+      <c r="AE7" t="n">
         <v>0.005</v>
       </c>
-      <c r="AE7" t="n">
+      <c r="AF7" t="n">
         <v>0.008399999999999999</v>
       </c>
-      <c r="AF7" t="n">
+      <c r="AG7" t="n">
         <v>0.0124</v>
       </c>
-      <c r="AG7" t="n">
+      <c r="AH7" t="n">
         <v>0.0187</v>
       </c>
-      <c r="AH7" t="n">
+      <c r="AI7" t="n">
         <v>0.008800000000000001</v>
       </c>
-      <c r="AI7" t="n">
+      <c r="AJ7" t="n">
         <v>0.0163</v>
       </c>
-      <c r="AJ7" t="n">
+      <c r="AK7" t="n">
         <v>0.0086</v>
       </c>
-      <c r="AK7" t="n">
+      <c r="AL7" t="n">
         <v>0.0067</v>
       </c>
-      <c r="AL7" t="n">
+      <c r="AM7" t="n">
         <v>153</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>성분</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>eye</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>EU_CLP</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>구조</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>338</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>116</v>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>0.3432</v>
       </c>
-      <c r="J8" t="n">
+      <c r="K8" t="n">
         <v>0.8013</v>
       </c>
-      <c r="K8" t="n">
+      <c r="L8" t="n">
         <v>0.0041</v>
       </c>
-      <c r="L8" t="n">
+      <c r="M8" t="n">
         <v>0.672</v>
       </c>
-      <c r="M8" t="n">
+      <c r="N8" t="n">
         <v>0.0074</v>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>0.6418</v>
       </c>
-      <c r="O8" t="n">
+      <c r="P8" t="n">
         <v>0.0155</v>
       </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
         <v>0.8252</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="R8" t="n">
         <v>0.7335</v>
       </c>
-      <c r="R8" t="n">
+      <c r="S8" t="n">
         <v>0.6729000000000001</v>
       </c>
-      <c r="S8" t="n">
+      <c r="T8" t="n">
         <v>0.6138</v>
       </c>
-      <c r="T8" t="n">
+      <c r="U8" t="n">
         <v>0.8441</v>
       </c>
-      <c r="U8" t="n">
+      <c r="V8" t="n">
         <v>0.4689</v>
       </c>
-      <c r="V8" t="n">
+      <c r="W8" t="n">
         <v>0.729</v>
       </c>
-      <c r="W8" t="n">
+      <c r="X8" t="n">
         <v>0.7651</v>
       </c>
-      <c r="X8" t="n">
+      <c r="Y8" t="n">
         <v>71.2</v>
       </c>
-      <c r="Y8" t="n">
+      <c r="Z8" t="n">
         <v>34.6</v>
       </c>
-      <c r="Z8" t="n">
+      <c r="AA8" t="n">
         <v>44.8</v>
       </c>
-      <c r="AA8" t="n">
+      <c r="AB8" t="n">
         <v>187.4</v>
       </c>
-      <c r="AB8" t="n">
+      <c r="AC8" t="n">
         <v>0.6923</v>
       </c>
-      <c r="AC8" t="n">
+      <c r="AD8" t="n">
         <v>0.373</v>
       </c>
-      <c r="AD8" t="n">
+      <c r="AE8" t="n">
         <v>0.0034</v>
       </c>
-      <c r="AE8" t="n">
+      <c r="AF8" t="n">
         <v>0.0092</v>
       </c>
-      <c r="AF8" t="n">
+      <c r="AG8" t="n">
         <v>0.0065</v>
       </c>
-      <c r="AG8" t="n">
+      <c r="AH8" t="n">
         <v>0.0261</v>
       </c>
-      <c r="AH8" t="n">
+      <c r="AI8" t="n">
         <v>0.0068</v>
       </c>
-      <c r="AI8" t="n">
+      <c r="AJ8" t="n">
         <v>0.0172</v>
       </c>
-      <c r="AJ8" t="n">
+      <c r="AK8" t="n">
         <v>0.0106</v>
       </c>
-      <c r="AK8" t="n">
+      <c r="AL8" t="n">
         <v>0.0061</v>
       </c>
-      <c r="AL8" t="n">
+      <c r="AM8" t="n">
         <v>153</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" t="n">
+        <v>0</v>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>성분</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>eye</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>EU_CLP</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>구조+지문</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>338</v>
       </c>
-      <c r="H9" t="n">
+      <c r="I9" t="n">
         <v>116</v>
       </c>
-      <c r="I9" t="n">
+      <c r="J9" t="n">
         <v>0.3432</v>
       </c>
-      <c r="J9" t="n">
+      <c r="K9" t="n">
         <v>0.804</v>
       </c>
-      <c r="K9" t="n">
+      <c r="L9" t="n">
         <v>0.0064</v>
       </c>
-      <c r="L9" t="n">
+      <c r="M9" t="n">
         <v>0.6714</v>
       </c>
-      <c r="M9" t="n">
+      <c r="N9" t="n">
         <v>0.0125</v>
       </c>
-      <c r="N9" t="n">
+      <c r="O9" t="n">
         <v>0.6193</v>
       </c>
-      <c r="O9" t="n">
+      <c r="P9" t="n">
         <v>0.0106</v>
       </c>
-      <c r="P9" t="n">
+      <c r="Q9" t="n">
         <v>0.8232</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="R9" t="n">
         <v>0.7213000000000001</v>
       </c>
-      <c r="R9" t="n">
+      <c r="S9" t="n">
         <v>0.6749000000000001</v>
       </c>
-      <c r="S9" t="n">
+      <c r="T9" t="n">
         <v>0.5724</v>
       </c>
-      <c r="T9" t="n">
+      <c r="U9" t="n">
         <v>0.8559</v>
       </c>
-      <c r="U9" t="n">
+      <c r="V9" t="n">
         <v>0.4476</v>
       </c>
-      <c r="V9" t="n">
+      <c r="W9" t="n">
         <v>0.7141</v>
       </c>
-      <c r="W9" t="n">
+      <c r="X9" t="n">
         <v>0.7586000000000001</v>
       </c>
-      <c r="X9" t="n">
+      <c r="Y9" t="n">
         <v>66.40000000000001</v>
       </c>
-      <c r="Y9" t="n">
+      <c r="Z9" t="n">
         <v>32</v>
       </c>
-      <c r="Z9" t="n">
+      <c r="AA9" t="n">
         <v>49.6</v>
       </c>
-      <c r="AA9" t="n">
+      <c r="AB9" t="n">
         <v>190</v>
       </c>
-      <c r="AB9" t="n">
+      <c r="AC9" t="n">
         <v>0.6947</v>
       </c>
-      <c r="AC9" t="n">
+      <c r="AD9" t="n">
         <v>0.325</v>
       </c>
-      <c r="AD9" t="n">
+      <c r="AE9" t="n">
         <v>0.0039</v>
       </c>
-      <c r="AE9" t="n">
+      <c r="AF9" t="n">
         <v>0.0068</v>
       </c>
-      <c r="AF9" t="n">
+      <c r="AG9" t="n">
         <v>0.01</v>
       </c>
-      <c r="AG9" t="n">
+      <c r="AH9" t="n">
         <v>0.0157</v>
       </c>
-      <c r="AH9" t="n">
+      <c r="AI9" t="n">
         <v>0.0071</v>
       </c>
-      <c r="AI9" t="n">
+      <c r="AJ9" t="n">
         <v>0.0131</v>
       </c>
-      <c r="AJ9" t="n">
+      <c r="AK9" t="n">
         <v>0.0071</v>
       </c>
-      <c r="AK9" t="n">
+      <c r="AL9" t="n">
         <v>0.0054</v>
       </c>
-      <c r="AL9" t="n">
+      <c r="AM9" t="n">
         <v>153</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" t="n">
+        <v>0</v>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>성분</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>skin</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>UN_GHS+EU_CLP+K_REACH+US_OSHA</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>구조</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>nan0</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>398</v>
       </c>
-      <c r="H10" t="n">
+      <c r="I10" t="n">
         <v>127</v>
       </c>
-      <c r="I10" t="n">
+      <c r="J10" t="n">
         <v>0.3191</v>
       </c>
-      <c r="J10" t="n">
+      <c r="K10" t="n">
         <v>0.7584</v>
       </c>
-      <c r="K10" t="n">
+      <c r="L10" t="n">
         <v>0.0047</v>
       </c>
-      <c r="L10" t="n">
+      <c r="M10" t="n">
         <v>0.5445</v>
       </c>
-      <c r="M10" t="n">
+      <c r="N10" t="n">
         <v>0.0103</v>
       </c>
-      <c r="N10" t="n">
+      <c r="O10" t="n">
         <v>0.5377999999999999</v>
       </c>
-      <c r="O10" t="n">
+      <c r="P10" t="n">
         <v>0.0297</v>
       </c>
-      <c r="P10" t="n">
+      <c r="Q10" t="n">
         <v>0.8053</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="R10" t="n">
         <v>0.6715</v>
       </c>
-      <c r="R10" t="n">
+      <c r="S10" t="n">
         <v>0.5822000000000001</v>
       </c>
-      <c r="S10" t="n">
+      <c r="T10" t="n">
         <v>0.5008</v>
       </c>
-      <c r="T10" t="n">
+      <c r="U10" t="n">
         <v>0.8317</v>
       </c>
-      <c r="U10" t="n">
+      <c r="V10" t="n">
         <v>0.3474</v>
       </c>
-      <c r="V10" t="n">
+      <c r="W10" t="n">
         <v>0.6663</v>
       </c>
-      <c r="W10" t="n">
+      <c r="X10" t="n">
         <v>0.7261</v>
       </c>
-      <c r="X10" t="n">
+      <c r="Y10" t="n">
         <v>63.6</v>
       </c>
-      <c r="Y10" t="n">
+      <c r="Z10" t="n">
         <v>45.6</v>
       </c>
-      <c r="Z10" t="n">
+      <c r="AA10" t="n">
         <v>63.4</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="AB10" t="n">
         <v>225.4</v>
       </c>
-      <c r="AB10" t="n">
+      <c r="AC10" t="n">
         <v>0.6364</v>
       </c>
-      <c r="AC10" t="n">
+      <c r="AD10" t="n">
         <v>0.385</v>
       </c>
-      <c r="AD10" t="n">
+      <c r="AE10" t="n">
         <v>0.0065</v>
       </c>
-      <c r="AE10" t="n">
+      <c r="AF10" t="n">
         <v>0.017</v>
       </c>
-      <c r="AF10" t="n">
+      <c r="AG10" t="n">
         <v>0.0177</v>
       </c>
-      <c r="AG10" t="n">
+      <c r="AH10" t="n">
         <v>0.0448</v>
       </c>
-      <c r="AH10" t="n">
+      <c r="AI10" t="n">
         <v>0.0142</v>
       </c>
-      <c r="AI10" t="n">
+      <c r="AJ10" t="n">
         <v>0.032</v>
       </c>
-      <c r="AJ10" t="n">
+      <c r="AK10" t="n">
         <v>0.0183</v>
       </c>
-      <c r="AK10" t="n">
+      <c r="AL10" t="n">
         <v>0.0105</v>
       </c>
-      <c r="AL10" t="n">
+      <c r="AM10" t="n">
         <v>168</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" t="n">
+        <v>0</v>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>성분</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>skin</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>UN_GHS+EU_CLP+K_REACH+US_OSHA</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>구조+지문</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>nan0</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>398</v>
       </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
         <v>127</v>
       </c>
-      <c r="I11" t="n">
+      <c r="J11" t="n">
         <v>0.3191</v>
       </c>
-      <c r="J11" t="n">
+      <c r="K11" t="n">
         <v>0.7762</v>
       </c>
-      <c r="K11" t="n">
+      <c r="L11" t="n">
         <v>0.0041</v>
       </c>
-      <c r="L11" t="n">
+      <c r="M11" t="n">
         <v>0.5655</v>
       </c>
-      <c r="M11" t="n">
+      <c r="N11" t="n">
         <v>0.0094</v>
       </c>
-      <c r="N11" t="n">
+      <c r="O11" t="n">
         <v>0.5683</v>
       </c>
-      <c r="O11" t="n">
+      <c r="P11" t="n">
         <v>0.0236</v>
       </c>
-      <c r="P11" t="n">
+      <c r="Q11" t="n">
         <v>0.8141</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="R11" t="n">
         <v>0.6912</v>
       </c>
-      <c r="R11" t="n">
+      <c r="S11" t="n">
         <v>0.6048</v>
       </c>
-      <c r="S11" t="n">
+      <c r="T11" t="n">
         <v>0.537</v>
       </c>
-      <c r="T11" t="n">
+      <c r="U11" t="n">
         <v>0.8354</v>
       </c>
-      <c r="U11" t="n">
+      <c r="V11" t="n">
         <v>0.3854</v>
       </c>
-      <c r="V11" t="n">
+      <c r="W11" t="n">
         <v>0.6862</v>
       </c>
-      <c r="W11" t="n">
+      <c r="X11" t="n">
         <v>0.7402</v>
       </c>
-      <c r="X11" t="n">
+      <c r="Y11" t="n">
         <v>68.2</v>
       </c>
-      <c r="Y11" t="n">
+      <c r="Z11" t="n">
         <v>44.6</v>
       </c>
-      <c r="Z11" t="n">
+      <c r="AA11" t="n">
         <v>58.8</v>
       </c>
-      <c r="AA11" t="n">
+      <c r="AB11" t="n">
         <v>226.4</v>
       </c>
-      <c r="AB11" t="n">
+      <c r="AC11" t="n">
         <v>0.6498</v>
       </c>
-      <c r="AC11" t="n">
+      <c r="AD11" t="n">
         <v>0.313</v>
       </c>
-      <c r="AD11" t="n">
+      <c r="AE11" t="n">
         <v>0.0064</v>
       </c>
-      <c r="AE11" t="n">
+      <c r="AF11" t="n">
         <v>0.0135</v>
       </c>
-      <c r="AF11" t="n">
+      <c r="AG11" t="n">
         <v>0.015</v>
       </c>
-      <c r="AG11" t="n">
+      <c r="AH11" t="n">
         <v>0.0391</v>
       </c>
-      <c r="AH11" t="n">
+      <c r="AI11" t="n">
         <v>0.0153</v>
       </c>
-      <c r="AI11" t="n">
+      <c r="AJ11" t="n">
         <v>0.0253</v>
       </c>
-      <c r="AJ11" t="n">
+      <c r="AK11" t="n">
         <v>0.0152</v>
       </c>
-      <c r="AK11" t="n">
+      <c r="AL11" t="n">
         <v>0.008999999999999999</v>
       </c>
-      <c r="AL11" t="n">
+      <c r="AM11" t="n">
         <v>168</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" t="n">
+        <v>0</v>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>성분</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>skin</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>UN_GHS+EU_CLP+K_REACH+US_OSHA</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>구조</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>398</v>
       </c>
-      <c r="H12" t="n">
+      <c r="I12" t="n">
         <v>127</v>
       </c>
-      <c r="I12" t="n">
+      <c r="J12" t="n">
         <v>0.3191</v>
       </c>
-      <c r="J12" t="n">
+      <c r="K12" t="n">
         <v>0.7586000000000001</v>
       </c>
-      <c r="K12" t="n">
+      <c r="L12" t="n">
         <v>0.0044</v>
       </c>
-      <c r="L12" t="n">
+      <c r="M12" t="n">
         <v>0.5458</v>
       </c>
-      <c r="M12" t="n">
+      <c r="N12" t="n">
         <v>0.008800000000000001</v>
       </c>
-      <c r="N12" t="n">
+      <c r="O12" t="n">
         <v>0.5495</v>
       </c>
-      <c r="O12" t="n">
+      <c r="P12" t="n">
         <v>0.0283</v>
       </c>
-      <c r="P12" t="n">
+      <c r="Q12" t="n">
         <v>0.8068</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="R12" t="n">
         <v>0.6782</v>
       </c>
-      <c r="R12" t="n">
+      <c r="S12" t="n">
         <v>0.5862000000000001</v>
       </c>
-      <c r="S12" t="n">
+      <c r="T12" t="n">
         <v>0.5181</v>
       </c>
-      <c r="T12" t="n">
+      <c r="U12" t="n">
         <v>0.8288</v>
       </c>
-      <c r="U12" t="n">
+      <c r="V12" t="n">
         <v>0.3593</v>
       </c>
-      <c r="V12" t="n">
+      <c r="W12" t="n">
         <v>0.6734</v>
       </c>
-      <c r="W12" t="n">
+      <c r="X12" t="n">
         <v>0.7296</v>
       </c>
-      <c r="X12" t="n">
+      <c r="Y12" t="n">
         <v>65.8</v>
       </c>
-      <c r="Y12" t="n">
+      <c r="Z12" t="n">
         <v>46.4</v>
       </c>
-      <c r="Z12" t="n">
+      <c r="AA12" t="n">
         <v>61.2</v>
       </c>
-      <c r="AA12" t="n">
+      <c r="AB12" t="n">
         <v>224.6</v>
       </c>
-      <c r="AB12" t="n">
+      <c r="AC12" t="n">
         <v>0.6411</v>
       </c>
-      <c r="AC12" t="n">
+      <c r="AD12" t="n">
         <v>0.384</v>
       </c>
-      <c r="AD12" t="n">
+      <c r="AE12" t="n">
         <v>0.0064</v>
       </c>
-      <c r="AE12" t="n">
+      <c r="AF12" t="n">
         <v>0.0165</v>
       </c>
-      <c r="AF12" t="n">
+      <c r="AG12" t="n">
         <v>0.0161</v>
       </c>
-      <c r="AG12" t="n">
+      <c r="AH12" t="n">
         <v>0.0418</v>
       </c>
-      <c r="AH12" t="n">
+      <c r="AI12" t="n">
         <v>0.0118</v>
       </c>
-      <c r="AI12" t="n">
+      <c r="AJ12" t="n">
         <v>0.0312</v>
       </c>
-      <c r="AJ12" t="n">
+      <c r="AK12" t="n">
         <v>0.0178</v>
       </c>
-      <c r="AK12" t="n">
+      <c r="AL12" t="n">
         <v>0.0105</v>
       </c>
-      <c r="AL12" t="n">
+      <c r="AM12" t="n">
         <v>168</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>성분</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>skin</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>UN_GHS+EU_CLP+K_REACH+US_OSHA</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>구조+지문</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>native</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>해당없음</t>
         </is>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>398</v>
       </c>
-      <c r="H13" t="n">
+      <c r="I13" t="n">
         <v>127</v>
       </c>
-      <c r="I13" t="n">
+      <c r="J13" t="n">
         <v>0.3191</v>
       </c>
-      <c r="J13" t="n">
+      <c r="K13" t="n">
         <v>0.7746</v>
       </c>
-      <c r="K13" t="n">
+      <c r="L13" t="n">
         <v>0.0045</v>
       </c>
-      <c r="L13" t="n">
+      <c r="M13" t="n">
         <v>0.5634</v>
       </c>
-      <c r="M13" t="n">
+      <c r="N13" t="n">
         <v>0.0102</v>
       </c>
-      <c r="N13" t="n">
+      <c r="O13" t="n">
         <v>0.5762</v>
       </c>
-      <c r="O13" t="n">
+      <c r="P13" t="n">
         <v>0.0299</v>
       </c>
-      <c r="P13" t="n">
+      <c r="Q13" t="n">
         <v>0.8162</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="R13" t="n">
         <v>0.6962</v>
       </c>
-      <c r="R13" t="n">
+      <c r="S13" t="n">
         <v>0.6091</v>
       </c>
-      <c r="S13" t="n">
+      <c r="T13" t="n">
         <v>0.548</v>
       </c>
-      <c r="T13" t="n">
+      <c r="U13" t="n">
         <v>0.8354</v>
       </c>
-      <c r="U13" t="n">
+      <c r="V13" t="n">
         <v>0.3951</v>
       </c>
-      <c r="V13" t="n">
+      <c r="W13" t="n">
         <v>0.6917</v>
       </c>
-      <c r="W13" t="n">
+      <c r="X13" t="n">
         <v>0.7437</v>
       </c>
-      <c r="X13" t="n">
+      <c r="Y13" t="n">
         <v>69.59999999999999</v>
       </c>
-      <c r="Y13" t="n">
+      <c r="Z13" t="n">
         <v>44.6</v>
       </c>
-      <c r="Z13" t="n">
+      <c r="AA13" t="n">
         <v>57.4</v>
       </c>
-      <c r="AA13" t="n">
+      <c r="AB13" t="n">
         <v>226.4</v>
       </c>
-      <c r="AB13" t="n">
+      <c r="AC13" t="n">
         <v>0.6429</v>
       </c>
-      <c r="AC13" t="n">
+      <c r="AD13" t="n">
         <v>0.319</v>
       </c>
-      <c r="AD13" t="n">
+      <c r="AE13" t="n">
         <v>0.004</v>
       </c>
-      <c r="AE13" t="n">
+      <c r="AF13" t="n">
         <v>0.0166</v>
       </c>
-      <c r="AF13" t="n">
+      <c r="AG13" t="n">
         <v>0.0092</v>
       </c>
-      <c r="AG13" t="n">
+      <c r="AH13" t="n">
         <v>0.049</v>
       </c>
-      <c r="AH13" t="n">
+      <c r="AI13" t="n">
         <v>0.0118</v>
       </c>
-      <c r="AI13" t="n">
+      <c r="AJ13" t="n">
         <v>0.0307</v>
       </c>
-      <c r="AJ13" t="n">
+      <c r="AK13" t="n">
         <v>0.0193</v>
       </c>
-      <c r="AK13" t="n">
+      <c r="AL13" t="n">
         <v>0.0089</v>
       </c>
-      <c r="AL13" t="n">
+      <c r="AM13" t="n">
         <v>168</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AL13"/>
+  <autoFilter ref="A1:AM13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>